<commit_message>
bronze-silver-gold, dbt 수정. bronze 데이터를 최대한 반영하도록.
</commit_message>
<xml_diff>
--- a/30_output_share/06_BRONZE노출감사.xlsx
+++ b/30_output_share/06_BRONZE노출감사.xlsx
@@ -5075,7 +5075,7 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>동명 GOLD 컬럼 존재</t>
+          <t>동명 GOLD 컬럼 + 실적재 projection 확인</t>
         </is>
       </c>
     </row>
@@ -6355,7 +6355,7 @@
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>동명 GOLD 컬럼 존재</t>
+          <t>동명 GOLD 컬럼 + 실적재 projection 확인</t>
         </is>
       </c>
     </row>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>동명 GOLD 컬럼 존재</t>
+          <t>동명 GOLD 컬럼 + 실적재 projection 확인</t>
         </is>
       </c>
     </row>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>동명 GOLD 컬럼 존재</t>
+          <t>동명 GOLD 컬럼 + 실적재 projection 확인</t>
         </is>
       </c>
     </row>
@@ -20657,7 +20657,7 @@
       </c>
       <c r="F433" s="11" t="inlineStr">
         <is>
-          <t>동명 GOLD 컬럼 존재</t>
+          <t>동명 GOLD 컬럼 + 실적재 projection 확인</t>
         </is>
       </c>
     </row>

</xml_diff>